<commit_message>
fix: sample Excel files and admission_year parsing for bulk upload
</commit_message>
<xml_diff>
--- a/backend/excel-files/sample_10_users.xlsx
+++ b/backend/excel-files/sample_10_users.xlsx
@@ -519,7 +519,7 @@
         <v>Accountant</v>
       </c>
       <c r="D7" t="str">
-        <v>Finance Office</v>
+        <v>School of Postgraduate Studies</v>
       </c>
       <c r="E7" t="str">
         <v>0244123467</v>
@@ -536,7 +536,7 @@
         <v>AccountingAssistant</v>
       </c>
       <c r="D8" t="str">
-        <v>Finance Office</v>
+        <v>School of Postgraduate Studies</v>
       </c>
       <c r="E8" t="str">
         <v>0244123484</v>

</xml_diff>

<commit_message>
fix: unique indexes (0301-0330) and emails for sample_30_students; unique names/emails for sample_10_users
</commit_message>
<xml_diff>
--- a/backend/excel-files/sample_10_users.xlsx
+++ b/backend/excel-files/sample_10_users.xlsx
@@ -425,10 +425,10 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Dr. John Mensah</v>
+        <v>Dr. Nana Wiredu</v>
       </c>
       <c r="B2" t="str">
-        <v>john.mensah@umat.edu.gh</v>
+        <v>nana.wiredu@umat.edu.gh</v>
       </c>
       <c r="C2" t="str">
         <v>Supervisor</v>
@@ -437,15 +437,15 @@
         <v>Computer Science and Engineering</v>
       </c>
       <c r="E2" t="str">
-        <v>0244123456</v>
+        <v>0244200101</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Prof. Grace Asante</v>
+        <v>Prof. Esi Turkson</v>
       </c>
       <c r="B3" t="str">
-        <v>grace.asante@umat.edu.gh</v>
+        <v>esi.turkson@umat.edu.gh</v>
       </c>
       <c r="C3" t="str">
         <v>Supervisor</v>
@@ -454,15 +454,15 @@
         <v>Electrical and Electronic Engineering</v>
       </c>
       <c r="E3" t="str">
-        <v>0244123457</v>
+        <v>0244200102</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Kwesi Adjei</v>
+        <v>Mansa Darko</v>
       </c>
       <c r="B4" t="str">
-        <v>kwesi.adjei@umat.edu.gh</v>
+        <v>mansa.darko@umat.edu.gh</v>
       </c>
       <c r="C4" t="str">
         <v>Admin</v>
@@ -471,15 +471,15 @@
         <v>School of Postgraduate Studies</v>
       </c>
       <c r="E4" t="str">
-        <v>0244123464</v>
+        <v>0244200103</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Efua Mensah</v>
+        <v>Kakra Tetteh</v>
       </c>
       <c r="B5" t="str">
-        <v>efua.mensah@umat.edu.gh</v>
+        <v>kakra.tetteh@umat.edu.gh</v>
       </c>
       <c r="C5" t="str">
         <v>Registrar</v>
@@ -488,15 +488,15 @@
         <v>School of Postgraduate Studies</v>
       </c>
       <c r="E5" t="str">
-        <v>0244123465</v>
+        <v>0244200104</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Peter Bonsu</v>
+        <v>Serwa Quaye</v>
       </c>
       <c r="B6" t="str">
-        <v>peter.bonsu@umat.edu.gh</v>
+        <v>serwa.quaye@umat.edu.gh</v>
       </c>
       <c r="C6" t="str">
         <v>ExamsOfficer</v>
@@ -505,15 +505,15 @@
         <v>School of Postgraduate Studies</v>
       </c>
       <c r="E6" t="str">
-        <v>0244123466</v>
+        <v>0244200105</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Adwoa Kwarteng</v>
+        <v>Ato Gyasi</v>
       </c>
       <c r="B7" t="str">
-        <v>adwoa.kwarteng@umat.edu.gh</v>
+        <v>ato.gyasi@umat.edu.gh</v>
       </c>
       <c r="C7" t="str">
         <v>Accountant</v>
@@ -522,15 +522,15 @@
         <v>School of Postgraduate Studies</v>
       </c>
       <c r="E7" t="str">
-        <v>0244123467</v>
+        <v>0244200106</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Daniel Frimpong</v>
+        <v>Araba Acquah</v>
       </c>
       <c r="B8" t="str">
-        <v>daniel.frimpong@umat.edu.gh</v>
+        <v>araba.acquah@umat.edu.gh</v>
       </c>
       <c r="C8" t="str">
         <v>AccountingAssistant</v>
@@ -539,49 +539,49 @@
         <v>School of Postgraduate Studies</v>
       </c>
       <c r="E8" t="str">
-        <v>0244123484</v>
+        <v>0244200107</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Prof. Kojo Nkrumah</v>
+        <v>Prof. Kodwo Poku</v>
       </c>
       <c r="B9" t="str">
-        <v>kojo.nkrumah@umat.edu.gh</v>
+        <v>kodwo.poku@umat.edu.gh</v>
       </c>
       <c r="C9" t="str">
         <v>Dean</v>
       </c>
       <c r="D9" t="str">
-        <v>Computer Science and Engineering</v>
+        <v>Mining Engineering</v>
       </c>
       <c r="E9" t="str">
-        <v>0244123468</v>
+        <v>0244200108</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Dr. Akua Sarpong</v>
+        <v>Dr. Panyin Asiedu</v>
       </c>
       <c r="B10" t="str">
-        <v>akua.sarpong@umat.edu.gh</v>
+        <v>panyin.asiedu@umat.edu.gh</v>
       </c>
       <c r="C10" t="str">
         <v>ViceDean</v>
       </c>
       <c r="D10" t="str">
-        <v>Electrical and Electronic Engineering</v>
+        <v>Geological Engineering</v>
       </c>
       <c r="E10" t="str">
-        <v>0244123469</v>
+        <v>0244200109</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Francis Ofosu</v>
+        <v>Ebo Nyarko</v>
       </c>
       <c r="B11" t="str">
-        <v>francis.ofosu@umat.edu.gh</v>
+        <v>ebo.nyarko@umat.edu.gh</v>
       </c>
       <c r="C11" t="str">
         <v>AdminAssistant</v>
@@ -590,7 +590,7 @@
         <v>School of Postgraduate Studies</v>
       </c>
       <c r="E11" t="str">
-        <v>0244123470</v>
+        <v>0244200110</v>
       </c>
     </row>
   </sheetData>

</xml_diff>